<commit_message>
Swap ID and item code columns in product list
Item code moves to column A and the ID to column B.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01CZxBBwADpmuwRLfknjnTgx
</commit_message>
<xml_diff>
--- a/tuco_kids_products.xlsx
+++ b/tuco_kids_products.xlsx
@@ -451,12 +451,12 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
+          <t>Item Code</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="inlineStr">
+        <is>
           <t>ID</t>
-        </is>
-      </c>
-      <c r="B1" s="2" t="inlineStr">
-        <is>
-          <t>Item Code</t>
         </is>
       </c>
       <c r="C1" s="2" t="inlineStr">
@@ -467,10 +467,10 @@
     </row>
     <row r="2">
       <c r="A2" s="3" t="n">
+        <v>1212203</v>
+      </c>
+      <c r="B2" s="3" t="n">
         <v>494846205</v>
-      </c>
-      <c r="B2" s="3" t="n">
-        <v>1212203</v>
       </c>
       <c r="C2" s="4" t="inlineStr">
         <is>
@@ -485,10 +485,10 @@
     </row>
     <row r="3">
       <c r="A3" s="3" t="n">
+        <v>1212202</v>
+      </c>
+      <c r="B3" s="3" t="n">
         <v>494846204</v>
-      </c>
-      <c r="B3" s="3" t="n">
-        <v>1212202</v>
       </c>
       <c r="C3" s="4" t="inlineStr">
         <is>
@@ -498,10 +498,10 @@
     </row>
     <row r="4">
       <c r="A4" s="3" t="n">
+        <v>1212201</v>
+      </c>
+      <c r="B4" s="3" t="n">
         <v>494846203</v>
-      </c>
-      <c r="B4" s="3" t="n">
-        <v>1212201</v>
       </c>
       <c r="C4" s="4" t="inlineStr">
         <is>
@@ -511,10 +511,10 @@
     </row>
     <row r="5">
       <c r="A5" s="3" t="n">
+        <v>1212200</v>
+      </c>
+      <c r="B5" s="3" t="n">
         <v>494846202</v>
-      </c>
-      <c r="B5" s="3" t="n">
-        <v>1212200</v>
       </c>
       <c r="C5" s="4" t="inlineStr">
         <is>
@@ -524,10 +524,10 @@
     </row>
     <row r="6">
       <c r="A6" s="3" t="n">
+        <v>1212199</v>
+      </c>
+      <c r="B6" s="3" t="n">
         <v>494846201</v>
-      </c>
-      <c r="B6" s="3" t="n">
-        <v>1212199</v>
       </c>
       <c r="C6" s="4" t="inlineStr">
         <is>

</xml_diff>